<commit_message>
Changes to tables to accomodate better ability handling
</commit_message>
<xml_diff>
--- a/Documentation/CRUD Table.xlsx
+++ b/Documentation/CRUD Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dyfry\workspace\2026\DAT602-Project\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84EE31D4-6995-4897-ACFE-69019B8FE272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE9E0C2-379C-483F-BB87-FCF181F317D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="86">
   <si>
     <t>Account</t>
   </si>
@@ -252,9 +252,6 @@
     <t>C__</t>
   </si>
   <si>
-    <t>AbilityName</t>
-  </si>
-  <si>
     <t>AbilityID (PK)</t>
   </si>
   <si>
@@ -271,6 +268,21 @@
   </si>
   <si>
     <t>StatisticName (PK) (FK)</t>
+  </si>
+  <si>
+    <t>AbilityName (PK)</t>
+  </si>
+  <si>
+    <t>Placed (PK)</t>
+  </si>
+  <si>
+    <t>Removed</t>
+  </si>
+  <si>
+    <t>AbilityInstance</t>
+  </si>
+  <si>
+    <t>AbilityName (FK)</t>
   </si>
 </sst>
 </file>
@@ -362,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -370,6 +382,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -650,7 +663,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T65"/>
+  <dimension ref="A1:T69"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.21875" customWidth="1"/>
@@ -2567,7 +2580,7 @@
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="B37" t="s">
         <v>65</v>
@@ -2691,7 +2704,7 @@
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B39" t="s">
         <v>65</v>
@@ -2752,94 +2765,94 @@
       </c>
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B40" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" t="s">
+        <v>65</v>
+      </c>
+      <c r="D40" t="s">
+        <v>65</v>
+      </c>
+      <c r="E40" t="s">
+        <v>65</v>
+      </c>
+      <c r="F40" t="s">
+        <v>65</v>
+      </c>
+      <c r="G40" t="s">
+        <v>65</v>
+      </c>
+      <c r="H40" t="s">
+        <v>64</v>
+      </c>
+      <c r="I40" t="s">
+        <v>69</v>
+      </c>
+      <c r="J40" t="s">
+        <v>65</v>
+      </c>
+      <c r="K40" t="s">
+        <v>65</v>
+      </c>
+      <c r="L40" t="s">
+        <v>65</v>
+      </c>
+      <c r="M40" t="s">
+        <v>68</v>
+      </c>
+      <c r="N40" t="s">
+        <v>70</v>
+      </c>
+      <c r="O40" t="s">
+        <v>65</v>
+      </c>
+      <c r="P40" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>65</v>
+      </c>
+      <c r="R40" t="s">
+        <v>64</v>
+      </c>
+      <c r="S40" t="s">
+        <v>65</v>
+      </c>
+      <c r="T40" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A41" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
-      <c r="L40" s="5"/>
-      <c r="M40" s="5"/>
-      <c r="N40" s="5"/>
-      <c r="O40" s="5"/>
-      <c r="P40" s="5"/>
-      <c r="Q40" s="5"/>
-      <c r="R40" s="5"/>
-      <c r="S40" s="5"/>
-      <c r="T40" s="5"/>
-    </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B41" t="s">
-        <v>65</v>
-      </c>
-      <c r="C41" t="s">
-        <v>65</v>
-      </c>
-      <c r="D41" t="s">
-        <v>65</v>
-      </c>
-      <c r="E41" t="s">
-        <v>65</v>
-      </c>
-      <c r="F41" t="s">
-        <v>65</v>
-      </c>
-      <c r="G41" t="s">
-        <v>68</v>
-      </c>
-      <c r="H41" t="s">
-        <v>65</v>
-      </c>
-      <c r="I41" t="s">
-        <v>64</v>
-      </c>
-      <c r="J41" t="s">
-        <v>64</v>
-      </c>
-      <c r="K41" t="s">
-        <v>65</v>
-      </c>
-      <c r="L41" t="s">
-        <v>65</v>
-      </c>
-      <c r="M41" t="s">
-        <v>65</v>
-      </c>
-      <c r="N41" t="s">
-        <v>65</v>
-      </c>
-      <c r="O41" t="s">
-        <v>65</v>
-      </c>
-      <c r="P41" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q41" t="s">
-        <v>65</v>
-      </c>
-      <c r="R41" t="s">
-        <v>64</v>
-      </c>
-      <c r="S41" t="s">
-        <v>65</v>
-      </c>
-      <c r="T41" t="s">
-        <v>65</v>
-      </c>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="K41" s="5"/>
+      <c r="L41" s="5"/>
+      <c r="M41" s="5"/>
+      <c r="N41" s="5"/>
+      <c r="O41" s="5"/>
+      <c r="P41" s="5"/>
+      <c r="Q41" s="5"/>
+      <c r="R41" s="5"/>
+      <c r="S41" s="5"/>
+      <c r="T41" s="5"/>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B42" t="s">
         <v>65</v>
@@ -3421,7 +3434,7 @@
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B52" t="s">
         <v>65</v>
@@ -3631,7 +3644,7 @@
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B56" t="s">
         <v>65</v>
@@ -3817,7 +3830,7 @@
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B59" s="5"/>
       <c r="C59" s="5"/>
@@ -3841,7 +3854,7 @@
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B60" t="s">
         <v>65</v>
@@ -3965,7 +3978,7 @@
     </row>
     <row r="62" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B62" s="5"/>
       <c r="C62" s="5"/>
@@ -3989,7 +4002,7 @@
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B63" t="s">
         <v>65</v>
@@ -4172,6 +4185,176 @@
       <c r="T65" t="s">
         <v>65</v>
       </c>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A66" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B66" s="5"/>
+      <c r="C66" s="5"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5"/>
+      <c r="H66" s="5"/>
+      <c r="I66" s="5"/>
+      <c r="J66" s="5"/>
+      <c r="K66" s="5"/>
+      <c r="L66" s="5"/>
+      <c r="M66" s="5"/>
+      <c r="N66" s="5"/>
+      <c r="O66" s="5"/>
+      <c r="P66" s="5"/>
+      <c r="Q66" s="5"/>
+      <c r="R66" s="5"/>
+      <c r="S66" s="5"/>
+      <c r="T66" s="5"/>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B67" t="s">
+        <v>65</v>
+      </c>
+      <c r="C67" t="s">
+        <v>65</v>
+      </c>
+      <c r="D67" t="s">
+        <v>65</v>
+      </c>
+      <c r="E67" t="s">
+        <v>65</v>
+      </c>
+      <c r="F67" t="s">
+        <v>65</v>
+      </c>
+      <c r="G67" t="s">
+        <v>65</v>
+      </c>
+      <c r="H67" t="s">
+        <v>64</v>
+      </c>
+      <c r="I67" t="s">
+        <v>64</v>
+      </c>
+      <c r="J67" t="s">
+        <v>64</v>
+      </c>
+      <c r="K67" t="s">
+        <v>65</v>
+      </c>
+      <c r="L67" t="s">
+        <v>65</v>
+      </c>
+      <c r="M67" t="s">
+        <v>65</v>
+      </c>
+      <c r="N67" t="s">
+        <v>70</v>
+      </c>
+      <c r="O67" t="s">
+        <v>65</v>
+      </c>
+      <c r="P67" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>65</v>
+      </c>
+      <c r="R67" t="s">
+        <v>64</v>
+      </c>
+      <c r="S67" t="s">
+        <v>65</v>
+      </c>
+      <c r="T67" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B68" t="s">
+        <v>65</v>
+      </c>
+      <c r="C68" t="s">
+        <v>65</v>
+      </c>
+      <c r="D68" t="s">
+        <v>65</v>
+      </c>
+      <c r="E68" t="s">
+        <v>65</v>
+      </c>
+      <c r="F68" t="s">
+        <v>65</v>
+      </c>
+      <c r="G68" t="s">
+        <v>65</v>
+      </c>
+      <c r="H68" t="s">
+        <v>64</v>
+      </c>
+      <c r="I68" t="s">
+        <v>64</v>
+      </c>
+      <c r="J68" t="s">
+        <v>64</v>
+      </c>
+      <c r="K68" t="s">
+        <v>65</v>
+      </c>
+      <c r="L68" t="s">
+        <v>65</v>
+      </c>
+      <c r="M68" t="s">
+        <v>65</v>
+      </c>
+      <c r="N68" t="s">
+        <v>70</v>
+      </c>
+      <c r="O68" t="s">
+        <v>65</v>
+      </c>
+      <c r="P68" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>65</v>
+      </c>
+      <c r="R68" t="s">
+        <v>64</v>
+      </c>
+      <c r="S68" t="s">
+        <v>65</v>
+      </c>
+      <c r="T68" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A69" s="7"/>
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="7"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="7"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="7"/>
+      <c r="I69" s="7"/>
+      <c r="J69" s="7"/>
+      <c r="K69" s="7"/>
+      <c r="L69" s="7"/>
+      <c r="M69" s="7"/>
+      <c r="N69" s="7"/>
+      <c r="O69" s="7"/>
+      <c r="P69" s="7"/>
+      <c r="Q69" s="7"/>
+      <c r="R69" s="7"/>
+      <c r="S69" s="7"/>
+      <c r="T69" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>